<commit_message>
fix(internal-quote): align archive, draft imports and quotation exports
</commit_message>
<xml_diff>
--- a/backend/app/data/internal_quote_import_templates/车缝报价单.xlsx
+++ b/backend/app/data/internal_quote_import_templates/车缝报价单.xlsx
@@ -1887,16 +1887,17 @@
     </x:row>
     <x:row r="10" s="41" customFormat="1" ht="48" customHeight="1">
       <x:c r="A10" s="55"/>
-      <x:c r="B10" s="65" t="s">
-        <x:v>17</x:v>
+      <x:c r="B10" s="65" t="str">
+        <x:f>'明细260707'!A2</x:f>
+        <x:v>8寸紫色土豆蝙蝠</x:v>
       </x:c>
       <x:c r="C10" s="66" t="n">
         <x:f>'明细260707'!K28</x:f>
         <x:v>41.90015081228894</x:v>
       </x:c>
-      <x:c r="D10" s="67" t="n">
-        <x:f t="shared" ref="D10:D15" si="0">C10*1.1</x:f>
-        <x:v>46.09016589351784</x:v>
+      <x:c r="D10" s="67">
+        <x:f>IF(C10="","",C10*1.1)</x:f>
+        <x:v>46.09016589351781</x:v>
       </x:c>
       <x:c r="E10" s="68"/>
       <x:c r="F10" s="69" t="s">
@@ -1909,16 +1910,11 @@
     </x:row>
     <x:row r="11" s="41" customFormat="1" ht="48" customHeight="1">
       <x:c r="A11" s="71"/>
-      <x:c r="B11" s="72" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C11" s="66" t="n">
-        <x:f>'明细260707'!K57</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D11" s="67">
-        <x:f t="shared" si="0"/>
-        <x:v>37.6907172148573</x:v>
+      <x:c r="B11" s="72"/>
+      <x:c r="C11" s="66"/>
+      <x:c r="D11" s="67" t="str">
+        <x:f>IF(C11="","",C11*1.1)</x:f>
+        <x:v/>
       </x:c>
       <x:c r="E11" s="68"/>
       <x:c r="F11" s="69"/>
@@ -1929,16 +1925,11 @@
     </x:row>
     <x:row r="12" s="41" customFormat="1" ht="48" customHeight="1">
       <x:c r="A12" s="55"/>
-      <x:c r="B12" s="73" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C12" s="47" t="n">
-        <x:f>'明细260707'!K86</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D12" s="67">
-        <x:f t="shared" si="0"/>
-        <x:v>38.5392529117673</x:v>
+      <x:c r="B12" s="73"/>
+      <x:c r="C12" s="47"/>
+      <x:c r="D12" s="67" t="str">
+        <x:f>IF(C12="","",C12*1.1)</x:f>
+        <x:v/>
       </x:c>
       <x:c r="E12" s="74"/>
       <x:c r="F12" s="69"/>
@@ -1949,16 +1940,11 @@
     </x:row>
     <x:row r="13" s="41" customFormat="1" ht="48" customHeight="1">
       <x:c r="A13" s="71"/>
-      <x:c r="B13" s="72" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="C13" s="75" t="n">
-        <x:f>'明细260707'!K111</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D13" s="67">
-        <x:f t="shared" si="0"/>
-        <x:v>37.0475795902773</x:v>
+      <x:c r="B13" s="72"/>
+      <x:c r="C13" s="75"/>
+      <x:c r="D13" s="67" t="str">
+        <x:f>IF(C13="","",C13*1.1)</x:f>
+        <x:v/>
       </x:c>
       <x:c r="E13" s="76"/>
       <x:c r="F13" s="77"/>
@@ -1969,16 +1955,11 @@
     </x:row>
     <x:row r="14" s="41" customFormat="1" ht="48" customHeight="1">
       <x:c r="A14" s="55"/>
-      <x:c r="B14" s="79" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="C14" s="66" t="n">
-        <x:f>'明细260707'!K137</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D14" s="67">
-        <x:f t="shared" si="0"/>
-        <x:v>37.6581438962773</x:v>
+      <x:c r="B14" s="79"/>
+      <x:c r="C14" s="66"/>
+      <x:c r="D14" s="67" t="str">
+        <x:f>IF(C14="","",C14*1.1)</x:f>
+        <x:v/>
       </x:c>
       <x:c r="E14" s="80"/>
       <x:c r="F14" s="69"/>
@@ -1989,16 +1970,11 @@
     </x:row>
     <x:row r="15" s="41" customFormat="1" ht="48" customHeight="1">
       <x:c r="A15" s="55"/>
-      <x:c r="B15" s="59" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C15" s="47" t="n">
-        <x:f>'明细260707'!K165</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D15" s="67">
-        <x:f t="shared" si="0"/>
-        <x:v>38.8137408164473</x:v>
+      <x:c r="B15" s="59"/>
+      <x:c r="C15" s="47"/>
+      <x:c r="D15" s="67" t="str">
+        <x:f>IF(C15="","",C15*1.1)</x:f>
+        <x:v/>
       </x:c>
       <x:c r="E15" s="55"/>
       <x:c r="F15" s="69"/>
@@ -2011,13 +1987,13 @@
       <x:c r="B16" s="81" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C16" s="82" t="n">
-        <x:f>AVERAGE(C10:C14)</x:f>
-        <x:v>8.380030162457789</x:v>
-      </x:c>
-      <x:c r="D16" s="82" t="n">
-        <x:f>AVERAGE(D10:D14)</x:f>
-        <x:v>39.405171901339415</x:v>
+      <x:c r="C16" s="82">
+        <x:f>SUM(C10:C15)</x:f>
+        <x:v>41.90015081228892</x:v>
+      </x:c>
+      <x:c r="D16" s="82">
+        <x:f>SUM(D10:D15)</x:f>
+        <x:v>46.09016589351781</x:v>
       </x:c>
       <x:c r="E16" s="47"/>
       <x:c r="F16" s="69"/>

</xml_diff>